<commit_message>
GL-4 DPE_GINI_P2 updated algorithm for FAM1_DIAB2
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
+++ b/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E838CA-3D7A-4A95-97D3-6DB7462FD167}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632AF36A-8C99-4887-8FCF-B7423CFC3BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22050" windowHeight="8100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1082,25 +1082,24 @@
     <t>Age at time of death [years]</t>
   </si>
   <si>
-    <t xml:space="preserve">If either parent has diabetes, the family history is marked as 1.
-If both parents do not have diabetes, the family history is marked as 0.                                                                                                                       If one parent's status is no or unknown (NA or 3), the family history is marked as 2. 
-If one parent's status is missing or unknown (NA or 3), the family history is marked as 2. </t>
+    <t>Sodium intake [mg/d]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sodium to potassium intake ratio </t>
   </si>
   <si>
     <t>case_when (
-  diabmut_15 == 1 | diabvat_15 == 1 ~ 1L,
-  diabmut_15 == 0 &amp; diabvat_15 == 0 ~ 0L,
-   diabmut_15 == 3 &amp; diabvat_15 == 0 ~ 2L,
-  diabvat_15 == 3 &amp; diabmut_15 == 0 ~ 2L,
-  (is.na(diabmut_15)  &amp;  diabvat_15 == 3 ~ 2L,                                                                          (is.na(diabvat_15)  &amp;  diabmut_15 == 3 ~ 2L, 
-  TRUE ~ NA_integer_
+      diabmut_15 == 1 | diabvat_15 == 1 ~ 1L,
+      diabmut_15 == 3 | diabvat_15 == 3 ~ 2L,
+      diabmut_15 == 2 &amp; diabvat_15 == 2 ~ 0L,
+      TRUE ~ NA_integer_
 )</t>
   </si>
   <si>
-    <t>Sodium intake [mg/d]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sodium to potassium intake ratio </t>
+    <t>If either parent has diabetes(1), the family history is marked as yes(1).
+If one parent's status is unknown (3), the family history is marked as don't know (2). 
+If both parents do not have diabetes (2), the family history is marked as no (0).
+Everything else (e.g. 2+ NA, NA+NA) is marked as NA</t>
   </si>
 </sst>
 </file>
@@ -2494,7 +2493,7 @@
       </c>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" s="5" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" s="5" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -2517,10 +2516,10 @@
         <v>27</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I29" s="18" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>29</v>
@@ -4533,7 +4532,7 @@
         <v>216</v>
       </c>
       <c r="C95" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D95" t="s">
         <v>22</v>
@@ -4566,7 +4565,7 @@
         <v>218</v>
       </c>
       <c r="C96" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D96" t="s">
         <v>22</v>
@@ -5089,27 +5088,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -5350,26 +5328,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
-    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2AE2FD3-517E-4530-8BC5-1FF35C67F615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5386,4 +5366,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
+    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
GL-4 DPE_GINI_P2 updated FAM_DIAB2 (need to update EDU_LEVEL)
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
+++ b/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632AF36A-8C99-4887-8FCF-B7423CFC3BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E42FA2B-B7B4-4F06-B7B4-ED3554A8C177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22260" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1090,16 +1090,16 @@
   <si>
     <t>case_when (
       diabmut_15 == 1 | diabvat_15 == 1 ~ 1L,
+      diabmut_15 == 2 | diabvat_15 == 2 ~ 0L,
       diabmut_15 == 3 | diabvat_15 == 3 ~ 2L,
-      diabmut_15 == 2 &amp; diabvat_15 == 2 ~ 0L,
       TRUE ~ NA_integer_
 )</t>
   </si>
   <si>
-    <t>If either parent has diabetes(1), the family history is marked as yes(1).
-If one parent's status is unknown (3), the family history is marked as don't know (2). 
-If both parents do not have diabetes (2), the family history is marked as no (0).
-Everything else (e.g. 2+ NA, NA+NA) is marked as NA</t>
+    <t>If either parent has diabetes (coded as 1), the family history is marked as Yes (1).
+If both parents do not have diabetes (coded as 2), and condition 1 does not apply, the family history is marked as No (0).
+If either parent's diabetes status is unknown (coded as 3), and conditions 1 and 2 do not apply, the family history is marked as Don't Know (2).
+All other cases are marked as NA.</t>
   </si>
 </sst>
 </file>
@@ -5088,6 +5088,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -5328,28 +5349,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
+    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2AE2FD3-517E-4530-8BC5-1FF35C67F615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5366,23 +5385,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
-    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
GL-4 DPE_GINI_P1+DPE_GINI_P2 updated EDU_LEVEL
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
+++ b/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E42FA2B-B7B4-4F06-B7B4-ED3554A8C177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C0FE36-616F-490D-8C17-6C549426E018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22260" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -111,14 +111,6 @@
     <t>case_when</t>
   </si>
   <si>
-    <t>If both gsc09m (mother) and gsc08v (father) are NA, assign 5L ("not specified").
-If one parent has "other degree" (5) and the other parent has a valid level, use the valid level.
-If both have "other degree" (5), assign 5L.
-If one parent is NA, use the other parent’s value and map it directly.
-Both Present: Use the maximum value between the two parents (pmax), then map it to the appropriate category.
-Default: Assign NA_integer_ for unexpected cases (should not occur).</t>
-  </si>
-  <si>
     <t>partial</t>
   </si>
   <si>
@@ -830,42 +822,6 @@
   </si>
   <si>
     <t>recode(1=1; 2= 0;  ELSE = NA)</t>
-  </si>
-  <si>
-    <t>case_when(
-      is.na(gsc09m) &amp; is.na(gsc08v) ~ 5L,
-      gsc09m == 5 &amp; !is.na(gsc08v) ~ case_when(
-        gsc08v == 6 ~ 0L,
-        gsc08v == 1 ~ 1L,
-        gsc08v == 2 ~ 2L,
-        gsc08v == 3 ~ 3L,
-        gsc08v &gt;= 4 ~ 4L
-      ),
-      gsc08v == 5 &amp; !is.na(gsc09m) ~ case_when(
-        gsc09m == 6 ~ 0L,
-        gsc09m == 1 ~ 1L,
-        gsc09m == 2 ~ 2L,
-        gsc09m == 3 ~ 3L,
-        gsc09m &gt;= 4 ~ 4L
-      ),
-      gsc09m == 5 &amp; gsc08v == 5 ~ 5L,
-      is.na(gsc09m) &amp; gsc08v == 6 ~ 0L,
-      is.na(gsc09m) &amp; gsc08v == 1 ~ 1L,
-      is.na(gsc09m) &amp; gsc08v == 2 ~ 2L,
-      is.na(gsc09m) &amp; gsc08v == 3 ~ 3L,
-      is.na(gsc09m) &amp; gsc08v &gt;= 4 ~ 4L,
-      is.na(gsc08v) &amp; gsc09m == 6 ~ 0L,
-      is.na(gsc08v) &amp; gsc09m == 1 ~ 1L,
-      is.na(gsc08v) &amp; gsc09m == 2 ~ 2L,
-      is.na(gsc08v) &amp; gsc09m == 3 ~ 3L,
-      is.na(gsc08v) &amp; gsc09m &gt;= 4 ~ 4L,
-      pmax(gsc09m, gsc08v, na.rm = TRUE) == 6 ~ 0L,
-      pmax(gsc09m, gsc08v, na.rm = TRUE) == 1 ~ 1L,
-      pmax(gsc09m, gsc08v, na.rm = TRUE) == 2 ~ 2L,
-      pmax(gsc09m, gsc08v, na.rm = TRUE) == 3 ~ 3L,
-      pmax(gsc09m, gsc08v, na.rm = TRUE) &gt;= 4 ~ 4L,
-      TRUE ~ NA_integer_
-    )</t>
   </si>
   <si>
     <t>case_when (
@@ -1100,6 +1056,47 @@
 If both parents do not have diabetes (coded as 2), and condition 1 does not apply, the family history is marked as No (0).
 If either parent's diabetes status is unknown (coded as 3), and conditions 1 and 2 do not apply, the family history is marked as Don't Know (2).
 All other cases are marked as NA.</t>
+  </si>
+  <si>
+    <t>case_when(
+  is.na(gsc09m) &amp; is.na(gsc08v) ~ NA_integer_,
+  gsc09m == 5 &amp; gsc08v == 5 ~ 5L,
+  gsc09m == 5 &amp; !is.na(gsc08v) ~ case_when(
+    gsc08v == 6 ~ 0L,
+    gsc08v %in% 1:3 ~ 3L,
+    gsc08v == 4 ~ 4L,
+    TRUE ~ 5L
+  ),
+  gsc08v == 5 &amp; !is.na(gsc09m) ~ case_when(
+    gsc09m == 6 ~ 0L,
+    gsc09m %in% 1:3 ~ 3L,
+    gsc09m == 4 ~ 4L,
+    TRUE ~ 5L
+  ),
+  gsc09m == 5 &amp; gsc08v != 5  ~ case_when(
+    gsc08v == 6 ~ 0L,
+    gsc08v %in% 1:3 ~ 3L,
+    gsc08v == 4 ~ 4L,
+    TRUE ~ 5L
+  ),
+  gsc08v == 5 &amp; gsc09m != 5  ~ case_when(
+    gsc09m == 6 ~ 0L,
+    gsc09m %in% 1:3 ~ 3L,
+    gsc09m == 4 ~ 4L,
+    TRUE ~ 5L
+  ),
+  gsc09m == 6 | gsc08v == 6  ~ 0L,
+  gsc09m %in% 1:3 | gsc08v %in% 1:3 ~ 3L,
+  gsc09m == 4 | gsc08v == 4 ~ 4L,
+  TRUE ~ 5L
+)</t>
+  </si>
+  <si>
+    <t>Missing values: If both gsc09m and gsc08v are missing, it returns NA.
+Both are "not specified": If both are 5, it returns 5.
+One is "not specified": If one of the variables is 5 (i.e., "Sonstiger Abschluss"), it uses the other parent’s value (if valid) to determine the education level.
+One is missing: If one of the parents has a missing value (NA), it checks the valid level of the other parent.
+Max of both: If neither is missing, it will return the highest level between both parents (0L for none, 3L for secondary school, 4L for longer education).</t>
   </si>
 </sst>
 </file>
@@ -1162,17 +1159,20 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1217,7 +1217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1267,6 +1267,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1597,7 +1600,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>0</v>
@@ -1704,7 +1707,7 @@
         <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -1726,7 +1729,7 @@
         <v>15</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
@@ -1751,17 +1754,17 @@
       <c r="G5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="I5" s="2" t="s">
+      <c r="H5" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:12" s="1" customFormat="1" ht="135" x14ac:dyDescent="0.25">
@@ -1769,10 +1772,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
         <v>31</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1781,22 +1784,22 @@
         <v>13</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>27</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="L6" s="2"/>
     </row>
@@ -1805,10 +1808,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
         <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
@@ -1817,22 +1820,22 @@
         <v>13</v>
       </c>
       <c r="F7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
         <v>37</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="I7" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="J7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" t="s">
         <v>29</v>
-      </c>
-      <c r="K7" t="s">
-        <v>30</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -1841,10 +1844,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -1853,19 +1856,19 @@
         <v>13</v>
       </c>
       <c r="F8" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="H8" s="20" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>15</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1873,10 +1876,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -1885,17 +1888,17 @@
         <v>13</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1903,10 +1906,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
         <v>48</v>
-      </c>
-      <c r="C10" t="s">
-        <v>49</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1915,19 +1918,19 @@
         <v>13</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1935,10 +1938,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -1947,16 +1950,16 @@
         <v>13</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1964,10 +1967,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
@@ -1976,16 +1979,16 @@
         <v>13</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1993,10 +1996,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -2005,16 +2008,16 @@
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2022,10 +2025,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
         <v>54</v>
-      </c>
-      <c r="C14" t="s">
-        <v>55</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -2034,22 +2037,22 @@
         <v>13</v>
       </c>
       <c r="F14" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2057,10 +2060,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>59</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -2070,19 +2073,19 @@
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I15" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2090,10 +2093,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" t="s">
         <v>62</v>
-      </c>
-      <c r="C16" t="s">
-        <v>63</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -2102,16 +2105,16 @@
         <v>13</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2119,10 +2122,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -2132,16 +2135,16 @@
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2149,10 +2152,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -2161,16 +2164,16 @@
         <v>13</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -2178,10 +2181,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -2190,16 +2193,16 @@
         <v>13</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -2207,19 +2210,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" t="s">
+        <v>277</v>
+      </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="C20" t="s">
-        <v>279</v>
-      </c>
-      <c r="D20" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>20</v>
@@ -2228,13 +2231,13 @@
         <v>20</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J20" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K20" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -2242,19 +2245,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" t="s">
+        <v>278</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="C21" t="s">
-        <v>280</v>
-      </c>
-      <c r="D21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>20</v>
@@ -2263,13 +2266,13 @@
         <v>20</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -2277,19 +2280,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" t="s">
+        <v>279</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="C22" t="s">
-        <v>281</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>73</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>20</v>
@@ -2298,13 +2301,13 @@
         <v>20</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J22" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -2312,19 +2315,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" t="s">
+        <v>280</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="C23" t="s">
-        <v>282</v>
-      </c>
-      <c r="D23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>20</v>
@@ -2333,13 +2336,13 @@
         <v>20</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J23" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -2347,10 +2350,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
         <v>76</v>
-      </c>
-      <c r="C24" t="s">
-        <v>77</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
@@ -2359,16 +2362,16 @@
         <v>13</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -2376,10 +2379,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" t="s">
         <v>78</v>
-      </c>
-      <c r="C25" t="s">
-        <v>79</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
@@ -2388,16 +2391,16 @@
         <v>13</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -2405,10 +2408,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
         <v>80</v>
-      </c>
-      <c r="C26" t="s">
-        <v>81</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
@@ -2417,16 +2420,16 @@
         <v>13</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2434,10 +2437,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" t="s">
         <v>82</v>
-      </c>
-      <c r="C27" t="s">
-        <v>83</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2446,19 +2449,19 @@
         <v>13</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>15</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2466,10 +2469,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" t="s">
         <v>85</v>
-      </c>
-      <c r="C28" t="s">
-        <v>86</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
@@ -2479,17 +2482,17 @@
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I28" s="8"/>
       <c r="J28" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M28" s="2"/>
     </row>
@@ -2498,10 +2501,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" t="s">
         <v>87</v>
-      </c>
-      <c r="C29" t="s">
-        <v>88</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -2510,22 +2513,22 @@
         <v>13</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G29" s="19" t="s">
         <v>27</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I29" s="18" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K29" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="M29" s="6"/>
     </row>
@@ -2534,10 +2537,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C30" t="s">
         <v>90</v>
-      </c>
-      <c r="C30" t="s">
-        <v>91</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
@@ -2547,16 +2550,16 @@
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -2564,10 +2567,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" t="s">
         <v>92</v>
-      </c>
-      <c r="C31" t="s">
-        <v>93</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
@@ -2576,16 +2579,16 @@
         <v>13</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -2593,10 +2596,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" t="s">
         <v>94</v>
-      </c>
-      <c r="C32" t="s">
-        <v>95</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
@@ -2605,16 +2608,16 @@
         <v>13</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2622,10 +2625,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" t="s">
         <v>96</v>
-      </c>
-      <c r="C33" t="s">
-        <v>97</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -2634,16 +2637,16 @@
         <v>13</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2651,10 +2654,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" t="s">
         <v>98</v>
-      </c>
-      <c r="C34" t="s">
-        <v>99</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
@@ -2663,16 +2666,16 @@
         <v>13</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2680,10 +2683,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C35" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
@@ -2692,16 +2695,16 @@
         <v>13</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2709,10 +2712,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C36" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
@@ -2721,16 +2724,16 @@
         <v>13</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2738,10 +2741,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C37" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
@@ -2750,16 +2753,16 @@
         <v>13</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2767,10 +2770,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>102</v>
+      </c>
+      <c r="C38" t="s">
         <v>103</v>
-      </c>
-      <c r="C38" t="s">
-        <v>104</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
@@ -2779,16 +2782,16 @@
         <v>13</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2796,10 +2799,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" t="s">
         <v>105</v>
-      </c>
-      <c r="C39" t="s">
-        <v>106</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
@@ -2808,16 +2811,16 @@
         <v>13</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2825,10 +2828,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" t="s">
         <v>107</v>
-      </c>
-      <c r="C40" t="s">
-        <v>108</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
@@ -2837,16 +2840,16 @@
         <v>13</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2854,10 +2857,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C41" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D41" t="s">
         <v>22</v>
@@ -2866,16 +2869,16 @@
         <v>13</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2883,10 +2886,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C42" t="s">
         <v>110</v>
-      </c>
-      <c r="C42" t="s">
-        <v>111</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
@@ -2895,16 +2898,16 @@
         <v>13</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -2912,10 +2915,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C43" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D43" t="s">
         <v>22</v>
@@ -2924,16 +2927,16 @@
         <v>13</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -2941,10 +2944,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>112</v>
+      </c>
+      <c r="C44" t="s">
         <v>113</v>
-      </c>
-      <c r="C44" t="s">
-        <v>114</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
@@ -2953,16 +2956,16 @@
         <v>13</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -2970,10 +2973,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C45" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D45" t="s">
         <v>22</v>
@@ -2982,16 +2985,16 @@
         <v>13</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -2999,10 +3002,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" t="s">
         <v>116</v>
-      </c>
-      <c r="C46" t="s">
-        <v>117</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
@@ -3011,16 +3014,16 @@
         <v>13</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -3028,10 +3031,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C47" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
@@ -3040,16 +3043,16 @@
         <v>13</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3057,10 +3060,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" t="s">
         <v>119</v>
-      </c>
-      <c r="C48" t="s">
-        <v>120</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
@@ -3069,16 +3072,16 @@
         <v>13</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -3086,10 +3089,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C49" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -3098,16 +3101,16 @@
         <v>13</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -3115,10 +3118,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C50" t="s">
         <v>122</v>
-      </c>
-      <c r="C50" t="s">
-        <v>123</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -3127,16 +3130,16 @@
         <v>13</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3144,10 +3147,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C51" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D51" t="s">
         <v>22</v>
@@ -3156,16 +3159,16 @@
         <v>13</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3173,10 +3176,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C52" t="s">
         <v>125</v>
-      </c>
-      <c r="C52" t="s">
-        <v>126</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
@@ -3185,16 +3188,16 @@
         <v>13</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -3202,10 +3205,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C53" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D53" t="s">
         <v>22</v>
@@ -3214,16 +3217,16 @@
         <v>13</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -3231,10 +3234,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C54" t="s">
         <v>128</v>
-      </c>
-      <c r="C54" t="s">
-        <v>129</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3243,16 +3246,16 @@
         <v>13</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -3260,10 +3263,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C55" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D55" t="s">
         <v>22</v>
@@ -3272,16 +3275,16 @@
         <v>13</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3289,10 +3292,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" t="s">
         <v>131</v>
-      </c>
-      <c r="C56" t="s">
-        <v>132</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
@@ -3301,16 +3304,16 @@
         <v>13</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -3318,10 +3321,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C57" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D57" t="s">
         <v>22</v>
@@ -3330,16 +3333,16 @@
         <v>13</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="58" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3347,10 +3350,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C58" t="s">
         <v>134</v>
-      </c>
-      <c r="C58" t="s">
-        <v>135</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -3360,16 +3363,16 @@
       </c>
       <c r="F58" s="13"/>
       <c r="G58" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -3377,28 +3380,28 @@
         <v>58</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C59" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D59" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3406,19 +3409,19 @@
         <v>59</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C60" t="s">
+        <v>320</v>
+      </c>
+      <c r="D60" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="C60" t="s">
-        <v>322</v>
-      </c>
-      <c r="D60" t="s">
-        <v>22</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>138</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>20</v>
@@ -3438,10 +3441,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C61" t="s">
         <v>139</v>
-      </c>
-      <c r="C61" t="s">
-        <v>140</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
@@ -3450,16 +3453,16 @@
         <v>13</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -3467,10 +3470,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C62" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -3479,16 +3482,16 @@
         <v>13</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3496,10 +3499,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C63" t="s">
         <v>142</v>
-      </c>
-      <c r="C63" t="s">
-        <v>143</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
@@ -3508,16 +3511,16 @@
         <v>13</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -3525,10 +3528,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C64" t="s">
         <v>144</v>
-      </c>
-      <c r="C64" t="s">
-        <v>145</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
@@ -3537,16 +3540,16 @@
         <v>13</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K64" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -3554,19 +3557,19 @@
         <v>64</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C65" t="s">
+        <v>285</v>
+      </c>
+      <c r="D65" t="s">
+        <v>22</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="7" t="s">
         <v>146</v>
-      </c>
-      <c r="C65" t="s">
-        <v>287</v>
-      </c>
-      <c r="D65" t="s">
-        <v>22</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F65" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>20</v>
@@ -3586,10 +3589,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C66" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D66" t="s">
         <v>22</v>
@@ -3598,7 +3601,7 @@
         <v>13</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G66" s="7" t="s">
         <v>20</v>
@@ -3619,10 +3622,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C67" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D67" t="s">
         <v>22</v>
@@ -3631,7 +3634,7 @@
         <v>13</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G67" s="7" t="s">
         <v>20</v>
@@ -3652,10 +3655,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C68" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
@@ -3664,7 +3667,7 @@
         <v>13</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>20</v>
@@ -3677,7 +3680,7 @@
         <v>15</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -3685,10 +3688,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C69" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
@@ -3698,17 +3701,17 @@
       </c>
       <c r="F69" s="9"/>
       <c r="G69" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I69"/>
       <c r="J69" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -3716,10 +3719,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C70" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D70" t="s">
         <v>22</v>
@@ -3729,17 +3732,17 @@
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H70" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I70" s="7"/>
       <c r="J70" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -3747,10 +3750,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C71" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D71" t="s">
         <v>22</v>
@@ -3760,17 +3763,17 @@
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I71" s="7"/>
       <c r="J71" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -3778,10 +3781,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C72" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D72" t="s">
         <v>22</v>
@@ -3791,17 +3794,17 @@
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H72" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I72" s="7"/>
       <c r="J72" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -3809,10 +3812,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C73" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D73" t="s">
         <v>22</v>
@@ -3822,17 +3825,17 @@
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I73" s="7"/>
       <c r="J73" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -3840,10 +3843,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C74" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D74" t="s">
         <v>22</v>
@@ -3853,17 +3856,17 @@
       </c>
       <c r="F74" s="7"/>
       <c r="G74" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H74" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I74" s="7"/>
       <c r="J74" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -3871,10 +3874,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C75" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D75" t="s">
         <v>22</v>
@@ -3883,7 +3886,7 @@
         <v>13</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="G75" s="7" t="s">
         <v>20</v>
@@ -3904,10 +3907,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C76" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D76" t="s">
         <v>22</v>
@@ -3917,17 +3920,17 @@
       </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H76" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I76" s="7"/>
       <c r="J76" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="77" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3935,19 +3938,19 @@
         <v>76</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C77" t="s">
+        <v>297</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" s="13" t="s">
         <v>159</v>
-      </c>
-      <c r="C77" t="s">
-        <v>299</v>
-      </c>
-      <c r="D77" t="s">
-        <v>22</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F77" s="13" t="s">
-        <v>160</v>
       </c>
       <c r="G77" s="7" t="s">
         <v>20</v>
@@ -3956,13 +3959,13 @@
         <v>20</v>
       </c>
       <c r="I77" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J77" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="78" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3970,10 +3973,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C78" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D78" t="s">
         <v>22</v>
@@ -3982,7 +3985,7 @@
         <v>13</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G78" s="7" t="s">
         <v>20</v>
@@ -4003,19 +4006,19 @@
         <v>78</v>
       </c>
       <c r="B79" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C79" t="s">
         <v>163</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
+        <v>22</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F79" s="7" t="s">
         <v>164</v>
-      </c>
-      <c r="D79" t="s">
-        <v>22</v>
-      </c>
-      <c r="E79" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F79" s="7" t="s">
-        <v>165</v>
       </c>
       <c r="G79" s="7" t="s">
         <v>20</v>
@@ -4036,25 +4039,25 @@
         <v>79</v>
       </c>
       <c r="B80" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C80" t="s">
         <v>166</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
+        <v>22</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F80" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="D80" t="s">
-        <v>22</v>
-      </c>
-      <c r="E80" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F80" s="7" t="s">
+      <c r="G80" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H80" s="7" t="s">
         <v>168</v>
-      </c>
-      <c r="G80" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H80" s="7" t="s">
-        <v>169</v>
       </c>
       <c r="I80" s="7"/>
       <c r="J80" s="7" t="s">
@@ -4069,25 +4072,25 @@
         <v>80</v>
       </c>
       <c r="B81" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C81" t="s">
         <v>170</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
+        <v>22</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F81" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="D81" t="s">
-        <v>22</v>
-      </c>
-      <c r="E81" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F81" s="7" t="s">
+      <c r="G81" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H81" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="G81" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H81" s="7" t="s">
-        <v>173</v>
       </c>
       <c r="I81" s="7"/>
       <c r="J81" s="7" t="s">
@@ -4102,25 +4105,25 @@
         <v>81</v>
       </c>
       <c r="B82" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C82" t="s">
         <v>174</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
+        <v>22</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F82" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="D82" t="s">
-        <v>22</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F82" s="7" t="s">
+      <c r="G82" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H82" s="7" t="s">
         <v>176</v>
-      </c>
-      <c r="G82" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H82" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="I82" s="7"/>
       <c r="J82" s="7" t="s">
@@ -4135,25 +4138,25 @@
         <v>82</v>
       </c>
       <c r="B83" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="C83" t="s">
         <v>178</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
+        <v>22</v>
+      </c>
+      <c r="E83" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F83" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D83" t="s">
-        <v>22</v>
-      </c>
-      <c r="E83" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F83" s="7" t="s">
+      <c r="G83" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H83" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="G83" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H83" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="I83" s="7"/>
       <c r="J83" s="7" t="s">
@@ -4168,25 +4171,25 @@
         <v>83</v>
       </c>
       <c r="B84" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C84" t="s">
         <v>182</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
+        <v>22</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F84" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D84" t="s">
-        <v>22</v>
-      </c>
-      <c r="E84" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F84" s="7" t="s">
+      <c r="G84" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H84" s="7" t="s">
         <v>184</v>
-      </c>
-      <c r="G84" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H84" s="7" t="s">
-        <v>185</v>
       </c>
       <c r="I84" s="7"/>
       <c r="J84" s="7" t="s">
@@ -4201,25 +4204,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C85" t="s">
         <v>186</v>
       </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
+        <v>22</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D85" t="s">
-        <v>22</v>
-      </c>
-      <c r="E85" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F85" s="7" t="s">
+      <c r="G85" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H85" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="G85" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H85" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="I85" s="7"/>
       <c r="J85" s="7" t="s">
@@ -4234,25 +4237,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="C86" t="s">
         <v>190</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
+        <v>22</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="D86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E86" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F86" s="7" t="s">
+      <c r="G86" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H86" s="7" t="s">
         <v>192</v>
-      </c>
-      <c r="G86" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H86" s="7" t="s">
-        <v>193</v>
       </c>
       <c r="I86" s="7"/>
       <c r="J86" s="7" t="s">
@@ -4267,25 +4270,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="C87" t="s">
         <v>194</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
+        <v>22</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="D87" t="s">
-        <v>22</v>
-      </c>
-      <c r="E87" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F87" s="7" t="s">
+      <c r="G87" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H87" s="7" t="s">
         <v>196</v>
-      </c>
-      <c r="G87" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H87" s="7" t="s">
-        <v>197</v>
       </c>
       <c r="I87" s="7"/>
       <c r="J87" s="7" t="s">
@@ -4300,10 +4303,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C88" t="s">
         <v>198</v>
-      </c>
-      <c r="C88" t="s">
-        <v>199</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -4313,17 +4316,17 @@
       </c>
       <c r="F88" s="7"/>
       <c r="G88" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H88" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I88" s="7"/>
       <c r="J88" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -4331,10 +4334,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="C89" t="s">
         <v>200</v>
-      </c>
-      <c r="C89" t="s">
-        <v>201</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -4344,17 +4347,17 @@
       </c>
       <c r="F89" s="7"/>
       <c r="G89" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H89" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I89" s="7"/>
       <c r="J89" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
@@ -4362,10 +4365,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C90" t="s">
         <v>202</v>
-      </c>
-      <c r="C90" t="s">
-        <v>203</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -4375,17 +4378,17 @@
       </c>
       <c r="F90" s="7"/>
       <c r="G90" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H90" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I90" s="7"/>
       <c r="J90" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
@@ -4393,25 +4396,25 @@
         <v>90</v>
       </c>
       <c r="B91" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="C91" t="s">
         <v>204</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
+        <v>22</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D91" t="s">
-        <v>22</v>
-      </c>
-      <c r="E91" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F91" s="7" t="s">
+      <c r="G91" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="G91" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H91" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="I91" s="7"/>
       <c r="J91" s="7" t="s">
@@ -4426,25 +4429,25 @@
         <v>91</v>
       </c>
       <c r="B92" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C92" t="s">
         <v>208</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
+        <v>22</v>
+      </c>
+      <c r="E92" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="D92" t="s">
-        <v>22</v>
-      </c>
-      <c r="E92" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F92" s="7" t="s">
+      <c r="G92" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H92" s="7" t="s">
         <v>210</v>
-      </c>
-      <c r="G92" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H92" s="7" t="s">
-        <v>211</v>
       </c>
       <c r="I92" s="7"/>
       <c r="J92" s="7" t="s">
@@ -4459,11 +4462,11 @@
         <v>92</v>
       </c>
       <c r="B93" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C93" t="s">
         <v>212</v>
       </c>
-      <c r="C93" t="s">
-        <v>213</v>
-      </c>
       <c r="D93" t="s">
         <v>22</v>
       </c>
@@ -4471,7 +4474,7 @@
         <v>13</v>
       </c>
       <c r="F93" s="13" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="G93" s="1" t="s">
         <v>20</v>
@@ -4480,7 +4483,7 @@
         <v>20</v>
       </c>
       <c r="I93" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J93" s="7" t="s">
         <v>15</v>
@@ -4494,10 +4497,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C94" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -4506,7 +4509,7 @@
         <v>13</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="G94" s="1" t="s">
         <v>20</v>
@@ -4515,7 +4518,7 @@
         <v>20</v>
       </c>
       <c r="I94" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J94" s="7" t="s">
         <v>15</v>
@@ -4529,19 +4532,19 @@
         <v>94</v>
       </c>
       <c r="B95" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C95" t="s">
+        <v>322</v>
+      </c>
+      <c r="D95" t="s">
+        <v>22</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" s="7" t="s">
         <v>216</v>
-      </c>
-      <c r="C95" t="s">
-        <v>324</v>
-      </c>
-      <c r="D95" t="s">
-        <v>22</v>
-      </c>
-      <c r="E95" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F95" s="7" t="s">
-        <v>217</v>
       </c>
       <c r="G95" s="1" t="s">
         <v>20</v>
@@ -4562,25 +4565,25 @@
         <v>95</v>
       </c>
       <c r="B96" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C96" t="s">
+        <v>323</v>
+      </c>
+      <c r="D96" t="s">
+        <v>22</v>
+      </c>
+      <c r="E96" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="C96" t="s">
-        <v>325</v>
-      </c>
-      <c r="D96" t="s">
-        <v>22</v>
-      </c>
-      <c r="E96" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F96" s="7" t="s">
+      <c r="G96" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H96" s="7" t="s">
         <v>219</v>
-      </c>
-      <c r="G96" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H96" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="I96" s="7"/>
       <c r="J96" s="7" t="s">
@@ -4595,32 +4598,32 @@
         <v>96</v>
       </c>
       <c r="B97" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C97" t="s">
         <v>221</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
+        <v>22</v>
+      </c>
+      <c r="E97" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H97" s="15" t="s">
         <v>222</v>
-      </c>
-      <c r="D97" t="s">
-        <v>22</v>
-      </c>
-      <c r="E97" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F97" s="15" t="s">
-        <v>307</v>
-      </c>
-      <c r="G97" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H97" s="15" t="s">
-        <v>223</v>
       </c>
       <c r="I97" s="7"/>
       <c r="J97" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K97" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="75" x14ac:dyDescent="0.25">
@@ -4628,10 +4631,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C98" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -4640,20 +4643,20 @@
         <v>13</v>
       </c>
       <c r="F98" s="15" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="G98" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H98" s="15" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I98" s="7"/>
       <c r="J98" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K98" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -4661,32 +4664,32 @@
         <v>98</v>
       </c>
       <c r="B99" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C99" t="s">
+        <v>301</v>
+      </c>
+      <c r="D99" t="s">
+        <v>22</v>
+      </c>
+      <c r="E99" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="C99" t="s">
-        <v>303</v>
-      </c>
-      <c r="D99" t="s">
-        <v>22</v>
-      </c>
-      <c r="E99" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" s="7" t="s">
+      <c r="G99" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H99" s="7" t="s">
         <v>226</v>
-      </c>
-      <c r="G99" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H99" s="7" t="s">
-        <v>227</v>
       </c>
       <c r="I99" s="7"/>
       <c r="J99" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -4694,32 +4697,32 @@
         <v>99</v>
       </c>
       <c r="B100" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="C100" t="s">
+        <v>302</v>
+      </c>
+      <c r="D100" t="s">
+        <v>22</v>
+      </c>
+      <c r="E100" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F100" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="C100" t="s">
-        <v>304</v>
-      </c>
-      <c r="D100" t="s">
-        <v>22</v>
-      </c>
-      <c r="E100" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F100" s="7" t="s">
+      <c r="G100" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H100" s="7" t="s">
         <v>229</v>
-      </c>
-      <c r="G100" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H100" s="7" t="s">
-        <v>230</v>
       </c>
       <c r="I100" s="7"/>
       <c r="J100" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K100" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
@@ -4727,10 +4730,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="C101" t="s">
         <v>231</v>
-      </c>
-      <c r="C101" t="s">
-        <v>232</v>
       </c>
       <c r="D101" t="s">
         <v>22</v>
@@ -4740,17 +4743,17 @@
       </c>
       <c r="F101" s="7"/>
       <c r="G101" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I101" s="7"/>
       <c r="J101" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K101" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -4758,32 +4761,32 @@
         <v>101</v>
       </c>
       <c r="B102" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C102" t="s">
         <v>233</v>
       </c>
-      <c r="C102" t="s">
+      <c r="D102" t="s">
+        <v>22</v>
+      </c>
+      <c r="E102" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="D102" t="s">
-        <v>22</v>
-      </c>
-      <c r="E102" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F102" s="7" t="s">
+      <c r="G102" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H102" s="7" t="s">
         <v>235</v>
-      </c>
-      <c r="G102" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H102" s="7" t="s">
-        <v>236</v>
       </c>
       <c r="I102" s="7"/>
       <c r="J102" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K102" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -4791,10 +4794,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C103" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D103" t="s">
         <v>22</v>
@@ -4804,17 +4807,17 @@
       </c>
       <c r="F103" s="7"/>
       <c r="G103" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H103" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I103" s="7"/>
       <c r="J103" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K103" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="60" x14ac:dyDescent="0.25">
@@ -4822,10 +4825,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C104" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D104" t="s">
         <v>22</v>
@@ -4834,20 +4837,20 @@
         <v>13</v>
       </c>
       <c r="F104" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H104" s="15" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="I104" s="7"/>
       <c r="J104" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K104" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -4855,11 +4858,11 @@
         <v>104</v>
       </c>
       <c r="B105" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C105" t="s">
         <v>239</v>
       </c>
-      <c r="C105" t="s">
-        <v>240</v>
-      </c>
       <c r="D105" t="s">
         <v>22</v>
       </c>
@@ -4867,20 +4870,20 @@
         <v>13</v>
       </c>
       <c r="F105" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G105" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H105" s="7" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I105" s="7"/>
       <c r="J105" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K105" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
@@ -4888,32 +4891,32 @@
         <v>105</v>
       </c>
       <c r="B106" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="C106" t="s">
         <v>241</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
+        <v>22</v>
+      </c>
+      <c r="E106" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F106" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="D106" t="s">
-        <v>22</v>
-      </c>
-      <c r="E106" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F106" s="7" t="s">
+      <c r="G106" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H106" s="7" t="s">
         <v>243</v>
-      </c>
-      <c r="G106" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H106" s="7" t="s">
-        <v>244</v>
       </c>
       <c r="I106" s="7"/>
       <c r="J106" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K106" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
@@ -4921,10 +4924,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C107" t="s">
         <v>245</v>
-      </c>
-      <c r="C107" t="s">
-        <v>246</v>
       </c>
       <c r="D107" t="s">
         <v>22</v>
@@ -4934,17 +4937,17 @@
       </c>
       <c r="F107" s="7"/>
       <c r="G107" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H107" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I107" s="7"/>
       <c r="J107" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -4952,19 +4955,19 @@
         <v>107</v>
       </c>
       <c r="B108" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="C108" t="s">
         <v>247</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D108" t="s">
+        <v>22</v>
+      </c>
+      <c r="E108" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F108" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="D108" t="s">
-        <v>22</v>
-      </c>
-      <c r="E108" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F108" s="7" t="s">
-        <v>249</v>
       </c>
       <c r="G108" s="7" t="s">
         <v>20</v>
@@ -4985,10 +4988,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
+        <v>249</v>
+      </c>
+      <c r="C109" t="s">
         <v>250</v>
-      </c>
-      <c r="C109" t="s">
-        <v>251</v>
       </c>
       <c r="D109" t="s">
         <v>12</v>
@@ -4997,16 +5000,16 @@
         <v>13</v>
       </c>
       <c r="F109" s="23" t="s">
+        <v>251</v>
+      </c>
+      <c r="G109" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="G109" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="H109">
         <v>1</v>
       </c>
       <c r="I109" s="24" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J109" s="12" t="s">
         <v>15</v>
@@ -5088,27 +5091,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -5349,26 +5331,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
-    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2AE2FD3-517E-4530-8BC5-1FF35C67F615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5385,4 +5369,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
+    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
GL-5 change in DPE + new mock data sets
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
+++ b/rmonize/data_proc_elem/DPE_GINI_P2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_proc_elem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C0FE36-616F-490D-8C17-6C549426E018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CC080C-5B3C-4740-A94E-9B52542DE142}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -105,9 +105,6 @@
     <t>Education</t>
   </si>
   <si>
-    <t>gsc09m; gsc08v</t>
-  </si>
-  <si>
     <t>case_when</t>
   </si>
   <si>
@@ -1059,44 +1056,23 @@
   </si>
   <si>
     <t>case_when(
-  is.na(gsc09m) &amp; is.na(gsc08v) ~ NA_integer_,
-  gsc09m == 5 &amp; gsc08v == 5 ~ 5L,
-  gsc09m == 5 &amp; !is.na(gsc08v) ~ case_when(
-    gsc08v == 6 ~ 0L,
-    gsc08v %in% 1:3 ~ 3L,
-    gsc08v == 4 ~ 4L,
-    TRUE ~ 5L
-  ),
-  gsc08v == 5 &amp; !is.na(gsc09m) ~ case_when(
-    gsc09m == 6 ~ 0L,
-    gsc09m %in% 1:3 ~ 3L,
-    gsc09m == 4 ~ 4L,
-    TRUE ~ 5L
-  ),
-  gsc09m == 5 &amp; gsc08v != 5  ~ case_when(
-    gsc08v == 6 ~ 0L,
-    gsc08v %in% 1:3 ~ 3L,
-    gsc08v == 4 ~ 4L,
-    TRUE ~ 5L
-  ),
-  gsc08v == 5 &amp; gsc09m != 5  ~ case_when(
-    gsc09m == 6 ~ 0L,
-    gsc09m %in% 1:3 ~ 3L,
-    gsc09m == 4 ~ 4L,
-    TRUE ~ 5L
-  ),
-  gsc09m == 6 | gsc08v == 6  ~ 0L,
-  gsc09m %in% 1:3 | gsc08v %in% 1:3 ~ 3L,
-  gsc09m == 4 | gsc08v == 4 ~ 4L,
-  TRUE ~ 5L
-)</t>
-  </si>
-  <si>
-    <t>Missing values: If both gsc09m and gsc08v are missing, it returns NA.
-Both are "not specified": If both are 5, it returns 5.
-One is "not specified": If one of the variables is 5 (i.e., "Sonstiger Abschluss"), it uses the other parent’s value (if valid) to determine the education level.
-One is missing: If one of the parents has a missing value (NA), it checks the valid level of the other parent.
-Max of both: If neither is missing, it will return the highest level between both parents (0L for none, 3L for secondary school, 4L for longer education).</t>
+  MUTBERU_3 %in% c(7) | VATBERU_3 %in% c(7) ~ 7L,
+  MUTBERU_3 %in% c(5,6) | VATBERU_3 %in% c(5,6) ~ 6L,
+  MUTBERU_3 %in% c(3,4) |VATBERU_3 %in% c(3,4) ~ 4L,
+  MUTBERU_3 %in% c(8) |VATBERU_3 %in% c(8) ~ 9L,
+  gsc09m %in% c(3) | gsc08v %in% c(3) ~ 3L,
+  gsc09m %in% c(1,2) | gsc08v %in% c(1,2) ~ 2L,
+  gsc09m %in% c(6) &amp; gsc08v %in% c(6) ~ 0L,
+  is.na(gsc09m) &amp; gsc08v %in% c(6) ~ 0L,
+  gsc09m %in% c(6) &amp; is.na(gsc08v) ~ 0L,
+  gsc09m %in% c(5) | gsc08v %in% c(5) ~ 9L,
+  TRUE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>gsc09m; gsc08v; MUTBERU_3; VATBERU_3</t>
+  </si>
+  <si>
+    <t>Education according to the ISCED 2011 classification</t>
   </si>
 </sst>
 </file>
@@ -1272,7 +1248,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1585,7 +1561,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M131"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="81.5703125" bestFit="1" customWidth="1"/>
@@ -1600,7 +1576,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>0</v>
@@ -1707,7 +1683,7 @@
         <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -1729,10 +1705,10 @@
         <v>15</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="1" customFormat="1" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1749,22 +1725,22 @@
         <v>13</v>
       </c>
       <c r="F5" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>27</v>
-      </c>
       <c r="H5" s="25" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="I5" s="16" t="s">
         <v>327</v>
       </c>
       <c r="J5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:12" s="1" customFormat="1" ht="135" x14ac:dyDescent="0.25">
@@ -1772,10 +1748,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1784,22 +1760,22 @@
         <v>13</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="I6" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="15" t="s">
-        <v>257</v>
-      </c>
-      <c r="I6" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="L6" s="2"/>
     </row>
@@ -1808,10 +1784,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
         <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
@@ -1820,22 +1796,22 @@
         <v>13</v>
       </c>
       <c r="F7" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s">
         <v>36</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="I7" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="I7" s="14" t="s">
-        <v>39</v>
-      </c>
       <c r="J7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" t="s">
         <v>28</v>
-      </c>
-      <c r="K7" t="s">
-        <v>29</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -1844,10 +1820,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -1856,19 +1832,19 @@
         <v>13</v>
       </c>
       <c r="F8" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="H8" s="20" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>15</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1876,10 +1852,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -1888,17 +1864,17 @@
         <v>13</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1906,10 +1882,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
         <v>47</v>
-      </c>
-      <c r="C10" t="s">
-        <v>48</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1918,19 +1894,19 @@
         <v>13</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1938,10 +1914,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -1950,16 +1926,16 @@
         <v>13</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1967,10 +1943,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
@@ -1979,16 +1955,16 @@
         <v>13</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1996,10 +1972,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -2008,16 +1984,16 @@
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2025,10 +2001,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
         <v>53</v>
-      </c>
-      <c r="C14" t="s">
-        <v>54</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -2037,22 +2013,22 @@
         <v>13</v>
       </c>
       <c r="F14" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2060,10 +2036,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" t="s">
         <v>57</v>
-      </c>
-      <c r="C15" t="s">
-        <v>58</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -2073,19 +2049,19 @@
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I15" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K15" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2093,10 +2069,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -2105,16 +2081,16 @@
         <v>13</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2122,10 +2098,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -2135,16 +2111,16 @@
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2152,10 +2128,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -2164,16 +2140,16 @@
         <v>13</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -2181,10 +2157,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C19" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -2193,16 +2169,16 @@
         <v>13</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -2210,19 +2186,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>276</v>
+      </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="C20" t="s">
-        <v>277</v>
-      </c>
-      <c r="D20" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>20</v>
@@ -2231,13 +2207,13 @@
         <v>20</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K20" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -2245,19 +2221,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
+        <v>277</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="C21" t="s">
-        <v>278</v>
-      </c>
-      <c r="D21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>20</v>
@@ -2266,13 +2242,13 @@
         <v>20</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -2280,19 +2256,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" t="s">
+        <v>278</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>71</v>
-      </c>
-      <c r="C22" t="s">
-        <v>279</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>72</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>20</v>
@@ -2301,13 +2277,13 @@
         <v>20</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -2315,19 +2291,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" t="s">
+        <v>279</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="C23" t="s">
-        <v>280</v>
-      </c>
-      <c r="D23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>74</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>20</v>
@@ -2336,13 +2312,13 @@
         <v>20</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -2350,10 +2326,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" t="s">
         <v>75</v>
-      </c>
-      <c r="C24" t="s">
-        <v>76</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
@@ -2362,16 +2338,16 @@
         <v>13</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -2379,10 +2355,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
         <v>77</v>
-      </c>
-      <c r="C25" t="s">
-        <v>78</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
@@ -2391,16 +2367,16 @@
         <v>13</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -2408,10 +2384,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" t="s">
         <v>79</v>
-      </c>
-      <c r="C26" t="s">
-        <v>80</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
@@ -2420,16 +2396,16 @@
         <v>13</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2437,10 +2413,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" t="s">
         <v>81</v>
-      </c>
-      <c r="C27" t="s">
-        <v>82</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2449,19 +2425,19 @@
         <v>13</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>15</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2469,10 +2445,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" t="s">
         <v>84</v>
-      </c>
-      <c r="C28" t="s">
-        <v>85</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
@@ -2482,17 +2458,17 @@
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I28" s="8"/>
       <c r="J28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M28" s="2"/>
     </row>
@@ -2501,10 +2477,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
         <v>86</v>
-      </c>
-      <c r="C29" t="s">
-        <v>87</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -2513,22 +2489,22 @@
         <v>13</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G29" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="J29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H29" s="17" t="s">
-        <v>324</v>
-      </c>
-      <c r="I29" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="J29" s="1" t="s">
+      <c r="K29" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="M29" s="6"/>
     </row>
@@ -2537,10 +2513,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" t="s">
         <v>89</v>
-      </c>
-      <c r="C30" t="s">
-        <v>90</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
@@ -2550,16 +2526,16 @@
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -2567,10 +2543,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" t="s">
         <v>91</v>
-      </c>
-      <c r="C31" t="s">
-        <v>92</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
@@ -2579,16 +2555,16 @@
         <v>13</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -2596,10 +2572,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" t="s">
         <v>93</v>
-      </c>
-      <c r="C32" t="s">
-        <v>94</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
@@ -2608,16 +2584,16 @@
         <v>13</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2625,10 +2601,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" t="s">
         <v>95</v>
-      </c>
-      <c r="C33" t="s">
-        <v>96</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -2637,16 +2613,16 @@
         <v>13</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2654,10 +2630,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" t="s">
         <v>97</v>
-      </c>
-      <c r="C34" t="s">
-        <v>98</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
@@ -2666,16 +2642,16 @@
         <v>13</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2683,10 +2659,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C35" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
@@ -2695,16 +2671,16 @@
         <v>13</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2712,10 +2688,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
@@ -2724,16 +2700,16 @@
         <v>13</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2741,10 +2717,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
@@ -2753,16 +2729,16 @@
         <v>13</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2770,10 +2746,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" t="s">
         <v>102</v>
-      </c>
-      <c r="C38" t="s">
-        <v>103</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
@@ -2782,16 +2758,16 @@
         <v>13</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2799,10 +2775,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>103</v>
+      </c>
+      <c r="C39" t="s">
         <v>104</v>
-      </c>
-      <c r="C39" t="s">
-        <v>105</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
@@ -2811,16 +2787,16 @@
         <v>13</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2828,10 +2804,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" t="s">
         <v>106</v>
-      </c>
-      <c r="C40" t="s">
-        <v>107</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
@@ -2840,16 +2816,16 @@
         <v>13</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2857,10 +2833,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C41" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D41" t="s">
         <v>22</v>
@@ -2869,16 +2845,16 @@
         <v>13</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2886,10 +2862,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" t="s">
         <v>109</v>
-      </c>
-      <c r="C42" t="s">
-        <v>110</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
@@ -2898,16 +2874,16 @@
         <v>13</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -2915,10 +2891,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C43" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D43" t="s">
         <v>22</v>
@@ -2927,16 +2903,16 @@
         <v>13</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -2944,10 +2920,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" t="s">
         <v>112</v>
-      </c>
-      <c r="C44" t="s">
-        <v>113</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
@@ -2956,16 +2932,16 @@
         <v>13</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -2973,10 +2949,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C45" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D45" t="s">
         <v>22</v>
@@ -2985,16 +2961,16 @@
         <v>13</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -3002,10 +2978,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C46" t="s">
         <v>115</v>
-      </c>
-      <c r="C46" t="s">
-        <v>116</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
@@ -3014,16 +2990,16 @@
         <v>13</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -3031,10 +3007,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C47" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
@@ -3043,16 +3019,16 @@
         <v>13</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3060,10 +3036,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C48" t="s">
         <v>118</v>
-      </c>
-      <c r="C48" t="s">
-        <v>119</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
@@ -3072,16 +3048,16 @@
         <v>13</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -3089,10 +3065,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C49" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -3101,16 +3077,16 @@
         <v>13</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -3118,10 +3094,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C50" t="s">
         <v>121</v>
-      </c>
-      <c r="C50" t="s">
-        <v>122</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -3130,16 +3106,16 @@
         <v>13</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3147,10 +3123,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C51" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D51" t="s">
         <v>22</v>
@@ -3159,16 +3135,16 @@
         <v>13</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3176,10 +3152,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C52" t="s">
         <v>124</v>
-      </c>
-      <c r="C52" t="s">
-        <v>125</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
@@ -3188,16 +3164,16 @@
         <v>13</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -3205,10 +3181,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C53" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D53" t="s">
         <v>22</v>
@@ -3217,16 +3193,16 @@
         <v>13</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -3234,10 +3210,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C54" t="s">
         <v>127</v>
-      </c>
-      <c r="C54" t="s">
-        <v>128</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3246,16 +3222,16 @@
         <v>13</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -3263,10 +3239,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C55" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D55" t="s">
         <v>22</v>
@@ -3275,16 +3251,16 @@
         <v>13</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3292,10 +3268,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>129</v>
+      </c>
+      <c r="C56" t="s">
         <v>130</v>
-      </c>
-      <c r="C56" t="s">
-        <v>131</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
@@ -3304,16 +3280,16 @@
         <v>13</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -3321,10 +3297,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C57" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D57" t="s">
         <v>22</v>
@@ -3333,16 +3309,16 @@
         <v>13</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="58" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3350,10 +3326,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C58" t="s">
         <v>133</v>
-      </c>
-      <c r="C58" t="s">
-        <v>134</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -3363,16 +3339,16 @@
       </c>
       <c r="F58" s="13"/>
       <c r="G58" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -3380,28 +3356,28 @@
         <v>58</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C59" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D59" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3409,19 +3385,19 @@
         <v>59</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C60" t="s">
+        <v>319</v>
+      </c>
+      <c r="D60" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="4" t="s">
         <v>136</v>
-      </c>
-      <c r="C60" t="s">
-        <v>320</v>
-      </c>
-      <c r="D60" t="s">
-        <v>22</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>137</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>20</v>
@@ -3441,10 +3417,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C61" t="s">
         <v>138</v>
-      </c>
-      <c r="C61" t="s">
-        <v>139</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
@@ -3453,16 +3429,16 @@
         <v>13</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -3470,10 +3446,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C62" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -3482,16 +3458,16 @@
         <v>13</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3499,10 +3475,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C63" t="s">
         <v>141</v>
-      </c>
-      <c r="C63" t="s">
-        <v>142</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
@@ -3511,16 +3487,16 @@
         <v>13</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -3528,10 +3504,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C64" t="s">
         <v>143</v>
-      </c>
-      <c r="C64" t="s">
-        <v>144</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
@@ -3540,16 +3516,16 @@
         <v>13</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K64" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -3557,19 +3533,19 @@
         <v>64</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C65" t="s">
+        <v>284</v>
+      </c>
+      <c r="D65" t="s">
+        <v>22</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="7" t="s">
         <v>145</v>
-      </c>
-      <c r="C65" t="s">
-        <v>285</v>
-      </c>
-      <c r="D65" t="s">
-        <v>22</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F65" s="7" t="s">
-        <v>146</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>20</v>
@@ -3589,10 +3565,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C66" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D66" t="s">
         <v>22</v>
@@ -3601,7 +3577,7 @@
         <v>13</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G66" s="7" t="s">
         <v>20</v>
@@ -3622,10 +3598,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C67" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D67" t="s">
         <v>22</v>
@@ -3634,7 +3610,7 @@
         <v>13</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G67" s="7" t="s">
         <v>20</v>
@@ -3655,10 +3631,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C68" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
@@ -3667,7 +3643,7 @@
         <v>13</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>20</v>
@@ -3680,7 +3656,7 @@
         <v>15</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="69" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -3688,10 +3664,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C69" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
@@ -3701,17 +3677,17 @@
       </c>
       <c r="F69" s="9"/>
       <c r="G69" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I69"/>
       <c r="J69" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -3719,10 +3695,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C70" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D70" t="s">
         <v>22</v>
@@ -3732,17 +3708,17 @@
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H70" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I70" s="7"/>
       <c r="J70" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -3750,10 +3726,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C71" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D71" t="s">
         <v>22</v>
@@ -3763,17 +3739,17 @@
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I71" s="7"/>
       <c r="J71" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -3781,10 +3757,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C72" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D72" t="s">
         <v>22</v>
@@ -3794,17 +3770,17 @@
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H72" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I72" s="7"/>
       <c r="J72" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -3812,10 +3788,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C73" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D73" t="s">
         <v>22</v>
@@ -3825,17 +3801,17 @@
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I73" s="7"/>
       <c r="J73" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -3843,10 +3819,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C74" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D74" t="s">
         <v>22</v>
@@ -3856,17 +3832,17 @@
       </c>
       <c r="F74" s="7"/>
       <c r="G74" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H74" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I74" s="7"/>
       <c r="J74" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -3874,10 +3850,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C75" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D75" t="s">
         <v>22</v>
@@ -3886,7 +3862,7 @@
         <v>13</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G75" s="7" t="s">
         <v>20</v>
@@ -3907,10 +3883,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C76" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D76" t="s">
         <v>22</v>
@@ -3920,17 +3896,17 @@
       </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H76" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I76" s="7"/>
       <c r="J76" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="77" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3938,19 +3914,19 @@
         <v>76</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C77" t="s">
+        <v>296</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" s="13" t="s">
         <v>158</v>
-      </c>
-      <c r="C77" t="s">
-        <v>297</v>
-      </c>
-      <c r="D77" t="s">
-        <v>22</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F77" s="13" t="s">
-        <v>159</v>
       </c>
       <c r="G77" s="7" t="s">
         <v>20</v>
@@ -3959,13 +3935,13 @@
         <v>20</v>
       </c>
       <c r="I77" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J77" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="78" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3973,10 +3949,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C78" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D78" t="s">
         <v>22</v>
@@ -3985,7 +3961,7 @@
         <v>13</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G78" s="7" t="s">
         <v>20</v>
@@ -4006,19 +3982,19 @@
         <v>78</v>
       </c>
       <c r="B79" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C79" t="s">
         <v>162</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
+        <v>22</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F79" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="D79" t="s">
-        <v>22</v>
-      </c>
-      <c r="E79" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F79" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="G79" s="7" t="s">
         <v>20</v>
@@ -4039,25 +4015,25 @@
         <v>79</v>
       </c>
       <c r="B80" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="C80" t="s">
         <v>165</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
+        <v>22</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F80" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D80" t="s">
-        <v>22</v>
-      </c>
-      <c r="E80" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F80" s="7" t="s">
+      <c r="G80" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H80" s="7" t="s">
         <v>167</v>
-      </c>
-      <c r="G80" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H80" s="7" t="s">
-        <v>168</v>
       </c>
       <c r="I80" s="7"/>
       <c r="J80" s="7" t="s">
@@ -4072,25 +4048,25 @@
         <v>80</v>
       </c>
       <c r="B81" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C81" t="s">
         <v>169</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
+        <v>22</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F81" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D81" t="s">
-        <v>22</v>
-      </c>
-      <c r="E81" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F81" s="7" t="s">
+      <c r="G81" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H81" s="7" t="s">
         <v>171</v>
-      </c>
-      <c r="G81" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H81" s="7" t="s">
-        <v>172</v>
       </c>
       <c r="I81" s="7"/>
       <c r="J81" s="7" t="s">
@@ -4105,25 +4081,25 @@
         <v>81</v>
       </c>
       <c r="B82" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C82" t="s">
         <v>173</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
+        <v>22</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F82" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="D82" t="s">
-        <v>22</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F82" s="7" t="s">
+      <c r="G82" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H82" s="7" t="s">
         <v>175</v>
-      </c>
-      <c r="G82" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H82" s="7" t="s">
-        <v>176</v>
       </c>
       <c r="I82" s="7"/>
       <c r="J82" s="7" t="s">
@@ -4138,25 +4114,25 @@
         <v>82</v>
       </c>
       <c r="B83" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C83" t="s">
         <v>177</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
+        <v>22</v>
+      </c>
+      <c r="E83" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F83" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="D83" t="s">
-        <v>22</v>
-      </c>
-      <c r="E83" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F83" s="7" t="s">
+      <c r="G83" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H83" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="G83" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H83" s="7" t="s">
-        <v>180</v>
       </c>
       <c r="I83" s="7"/>
       <c r="J83" s="7" t="s">
@@ -4171,25 +4147,25 @@
         <v>83</v>
       </c>
       <c r="B84" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C84" t="s">
         <v>181</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
+        <v>22</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F84" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="D84" t="s">
-        <v>22</v>
-      </c>
-      <c r="E84" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F84" s="7" t="s">
+      <c r="G84" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H84" s="7" t="s">
         <v>183</v>
-      </c>
-      <c r="G84" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H84" s="7" t="s">
-        <v>184</v>
       </c>
       <c r="I84" s="7"/>
       <c r="J84" s="7" t="s">
@@ -4204,25 +4180,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C85" t="s">
         <v>185</v>
       </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
+        <v>22</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D85" t="s">
-        <v>22</v>
-      </c>
-      <c r="E85" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F85" s="7" t="s">
+      <c r="G85" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H85" s="7" t="s">
         <v>187</v>
-      </c>
-      <c r="G85" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H85" s="7" t="s">
-        <v>188</v>
       </c>
       <c r="I85" s="7"/>
       <c r="J85" s="7" t="s">
@@ -4237,25 +4213,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C86" t="s">
         <v>189</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
+        <v>22</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="D86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E86" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F86" s="7" t="s">
+      <c r="G86" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H86" s="7" t="s">
         <v>191</v>
-      </c>
-      <c r="G86" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H86" s="7" t="s">
-        <v>192</v>
       </c>
       <c r="I86" s="7"/>
       <c r="J86" s="7" t="s">
@@ -4270,25 +4246,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C87" t="s">
         <v>193</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
+        <v>22</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="D87" t="s">
-        <v>22</v>
-      </c>
-      <c r="E87" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F87" s="7" t="s">
+      <c r="G87" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H87" s="7" t="s">
         <v>195</v>
-      </c>
-      <c r="G87" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H87" s="7" t="s">
-        <v>196</v>
       </c>
       <c r="I87" s="7"/>
       <c r="J87" s="7" t="s">
@@ -4303,10 +4279,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C88" t="s">
         <v>197</v>
-      </c>
-      <c r="C88" t="s">
-        <v>198</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -4316,17 +4292,17 @@
       </c>
       <c r="F88" s="7"/>
       <c r="G88" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H88" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I88" s="7"/>
       <c r="J88" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -4334,10 +4310,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C89" t="s">
         <v>199</v>
-      </c>
-      <c r="C89" t="s">
-        <v>200</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -4347,17 +4323,17 @@
       </c>
       <c r="F89" s="7"/>
       <c r="G89" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H89" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I89" s="7"/>
       <c r="J89" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
@@ -4365,10 +4341,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C90" t="s">
         <v>201</v>
-      </c>
-      <c r="C90" t="s">
-        <v>202</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -4378,17 +4354,17 @@
       </c>
       <c r="F90" s="7"/>
       <c r="G90" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H90" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I90" s="7"/>
       <c r="J90" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
@@ -4396,25 +4372,25 @@
         <v>90</v>
       </c>
       <c r="B91" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C91" t="s">
         <v>203</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
+        <v>22</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D91" t="s">
-        <v>22</v>
-      </c>
-      <c r="E91" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F91" s="7" t="s">
+      <c r="G91" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>205</v>
-      </c>
-      <c r="G91" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H91" s="7" t="s">
-        <v>206</v>
       </c>
       <c r="I91" s="7"/>
       <c r="J91" s="7" t="s">
@@ -4429,25 +4405,25 @@
         <v>91</v>
       </c>
       <c r="B92" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="C92" t="s">
         <v>207</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
+        <v>22</v>
+      </c>
+      <c r="E92" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D92" t="s">
-        <v>22</v>
-      </c>
-      <c r="E92" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F92" s="7" t="s">
+      <c r="G92" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H92" s="7" t="s">
         <v>209</v>
-      </c>
-      <c r="G92" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H92" s="7" t="s">
-        <v>210</v>
       </c>
       <c r="I92" s="7"/>
       <c r="J92" s="7" t="s">
@@ -4462,11 +4438,11 @@
         <v>92</v>
       </c>
       <c r="B93" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="C93" t="s">
         <v>211</v>
       </c>
-      <c r="C93" t="s">
-        <v>212</v>
-      </c>
       <c r="D93" t="s">
         <v>22</v>
       </c>
@@ -4474,7 +4450,7 @@
         <v>13</v>
       </c>
       <c r="F93" s="13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G93" s="1" t="s">
         <v>20</v>
@@ -4483,7 +4459,7 @@
         <v>20</v>
       </c>
       <c r="I93" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J93" s="7" t="s">
         <v>15</v>
@@ -4497,10 +4473,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C94" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D94" t="s">
         <v>22</v>
@@ -4509,7 +4485,7 @@
         <v>13</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G94" s="1" t="s">
         <v>20</v>
@@ -4518,7 +4494,7 @@
         <v>20</v>
       </c>
       <c r="I94" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J94" s="7" t="s">
         <v>15</v>
@@ -4532,19 +4508,19 @@
         <v>94</v>
       </c>
       <c r="B95" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C95" t="s">
+        <v>321</v>
+      </c>
+      <c r="D95" t="s">
+        <v>22</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" s="7" t="s">
         <v>215</v>
-      </c>
-      <c r="C95" t="s">
-        <v>322</v>
-      </c>
-      <c r="D95" t="s">
-        <v>22</v>
-      </c>
-      <c r="E95" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F95" s="7" t="s">
-        <v>216</v>
       </c>
       <c r="G95" s="1" t="s">
         <v>20</v>
@@ -4565,25 +4541,25 @@
         <v>95</v>
       </c>
       <c r="B96" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C96" t="s">
+        <v>322</v>
+      </c>
+      <c r="D96" t="s">
+        <v>22</v>
+      </c>
+      <c r="E96" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="C96" t="s">
-        <v>323</v>
-      </c>
-      <c r="D96" t="s">
-        <v>22</v>
-      </c>
-      <c r="E96" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F96" s="7" t="s">
+      <c r="G96" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H96" s="7" t="s">
         <v>218</v>
-      </c>
-      <c r="G96" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H96" s="7" t="s">
-        <v>219</v>
       </c>
       <c r="I96" s="7"/>
       <c r="J96" s="7" t="s">
@@ -4598,32 +4574,32 @@
         <v>96</v>
       </c>
       <c r="B97" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="C97" t="s">
         <v>220</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
+        <v>22</v>
+      </c>
+      <c r="E97" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H97" s="15" t="s">
         <v>221</v>
-      </c>
-      <c r="D97" t="s">
-        <v>22</v>
-      </c>
-      <c r="E97" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F97" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="G97" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H97" s="15" t="s">
-        <v>222</v>
       </c>
       <c r="I97" s="7"/>
       <c r="J97" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K97" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="75" x14ac:dyDescent="0.25">
@@ -4631,10 +4607,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C98" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D98" t="s">
         <v>22</v>
@@ -4643,20 +4619,20 @@
         <v>13</v>
       </c>
       <c r="F98" s="15" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G98" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H98" s="15" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I98" s="7"/>
       <c r="J98" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K98" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -4664,32 +4640,32 @@
         <v>98</v>
       </c>
       <c r="B99" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C99" t="s">
+        <v>300</v>
+      </c>
+      <c r="D99" t="s">
+        <v>22</v>
+      </c>
+      <c r="E99" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="C99" t="s">
-        <v>301</v>
-      </c>
-      <c r="D99" t="s">
-        <v>22</v>
-      </c>
-      <c r="E99" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" s="7" t="s">
+      <c r="G99" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H99" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="G99" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H99" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="I99" s="7"/>
       <c r="J99" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -4697,32 +4673,32 @@
         <v>99</v>
       </c>
       <c r="B100" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C100" t="s">
+        <v>301</v>
+      </c>
+      <c r="D100" t="s">
+        <v>22</v>
+      </c>
+      <c r="E100" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F100" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="C100" t="s">
-        <v>302</v>
-      </c>
-      <c r="D100" t="s">
-        <v>22</v>
-      </c>
-      <c r="E100" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F100" s="7" t="s">
+      <c r="G100" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H100" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="G100" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H100" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="I100" s="7"/>
       <c r="J100" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K100" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
@@ -4730,10 +4706,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="C101" t="s">
         <v>230</v>
-      </c>
-      <c r="C101" t="s">
-        <v>231</v>
       </c>
       <c r="D101" t="s">
         <v>22</v>
@@ -4743,17 +4719,17 @@
       </c>
       <c r="F101" s="7"/>
       <c r="G101" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I101" s="7"/>
       <c r="J101" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K101" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -4761,32 +4737,32 @@
         <v>101</v>
       </c>
       <c r="B102" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C102" t="s">
         <v>232</v>
       </c>
-      <c r="C102" t="s">
+      <c r="D102" t="s">
+        <v>22</v>
+      </c>
+      <c r="E102" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="D102" t="s">
-        <v>22</v>
-      </c>
-      <c r="E102" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F102" s="7" t="s">
+      <c r="G102" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H102" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="G102" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H102" s="7" t="s">
-        <v>235</v>
       </c>
       <c r="I102" s="7"/>
       <c r="J102" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K102" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -4794,10 +4770,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D103" t="s">
         <v>22</v>
@@ -4807,17 +4783,17 @@
       </c>
       <c r="F103" s="7"/>
       <c r="G103" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H103" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I103" s="7"/>
       <c r="J103" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K103" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="60" x14ac:dyDescent="0.25">
@@ -4825,10 +4801,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C104" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D104" t="s">
         <v>22</v>
@@ -4837,20 +4813,20 @@
         <v>13</v>
       </c>
       <c r="F104" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H104" s="15" t="s">
         <v>258</v>
-      </c>
-      <c r="G104" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H104" s="15" t="s">
-        <v>259</v>
       </c>
       <c r="I104" s="7"/>
       <c r="J104" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K104" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -4858,11 +4834,11 @@
         <v>104</v>
       </c>
       <c r="B105" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C105" t="s">
         <v>238</v>
       </c>
-      <c r="C105" t="s">
-        <v>239</v>
-      </c>
       <c r="D105" t="s">
         <v>22</v>
       </c>
@@ -4870,20 +4846,20 @@
         <v>13</v>
       </c>
       <c r="F105" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="G105" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H105" s="7" t="s">
         <v>260</v>
-      </c>
-      <c r="G105" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H105" s="7" t="s">
-        <v>261</v>
       </c>
       <c r="I105" s="7"/>
       <c r="J105" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K105" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
@@ -4891,32 +4867,32 @@
         <v>105</v>
       </c>
       <c r="B106" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C106" t="s">
         <v>240</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
+        <v>22</v>
+      </c>
+      <c r="E106" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F106" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="D106" t="s">
-        <v>22</v>
-      </c>
-      <c r="E106" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F106" s="7" t="s">
+      <c r="G106" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H106" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="G106" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H106" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="I106" s="7"/>
       <c r="J106" s="7" t="s">
         <v>15</v>
       </c>
       <c r="K106" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
@@ -4924,10 +4900,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C107" t="s">
         <v>244</v>
-      </c>
-      <c r="C107" t="s">
-        <v>245</v>
       </c>
       <c r="D107" t="s">
         <v>22</v>
@@ -4937,17 +4913,17 @@
       </c>
       <c r="F107" s="7"/>
       <c r="G107" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H107" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I107" s="7"/>
       <c r="J107" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -4955,19 +4931,19 @@
         <v>107</v>
       </c>
       <c r="B108" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="C108" t="s">
         <v>246</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D108" t="s">
+        <v>22</v>
+      </c>
+      <c r="E108" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F108" s="7" t="s">
         <v>247</v>
-      </c>
-      <c r="D108" t="s">
-        <v>22</v>
-      </c>
-      <c r="E108" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F108" s="7" t="s">
-        <v>248</v>
       </c>
       <c r="G108" s="7" t="s">
         <v>20</v>
@@ -4988,10 +4964,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
+        <v>248</v>
+      </c>
+      <c r="C109" t="s">
         <v>249</v>
-      </c>
-      <c r="C109" t="s">
-        <v>250</v>
       </c>
       <c r="D109" t="s">
         <v>12</v>
@@ -5000,16 +4976,16 @@
         <v>13</v>
       </c>
       <c r="F109" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="G109" s="3" t="s">
         <v>251</v>
-      </c>
-      <c r="G109" s="3" t="s">
-        <v>252</v>
       </c>
       <c r="H109">
         <v>1</v>
       </c>
       <c r="I109" s="24" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J109" s="12" t="s">
         <v>15</v>
@@ -5091,6 +5067,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -5331,7 +5319,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -5340,19 +5328,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
+    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2AE2FD3-517E-4530-8BC5-1FF35C67F615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5371,21 +5358,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CA3EE-638E-435F-8CA6-D67A7B863103}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADF2265-5030-4B54-A34F-4798AFD4DA4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
-    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>